<commit_message>
Add FY2025 vs FY2024 variance analysis with volume/rate split and deficit bridge
</commit_message>
<xml_diff>
--- a/excel-model/CIS_Chicago_FPA_Model.xlsx
+++ b/excel-model/CIS_Chicago_FPA_Model.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Inputs" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Historical" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Forecast" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Variance" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Forecast" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Scenarios" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Dashboard!$A$1:$M$58</definedName>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="394">
   <si>
     <t xml:space="preserve">Funding Shock Stress Test: Communities In Schools of Chicago</t>
   </si>
@@ -692,6 +693,135 @@
     <t xml:space="preserve">Gap between these = size of the swing</t>
   </si>
   <si>
+    <t xml:space="preserve">Variance analysis - FY2025 actual vs FY2024 actual  |  CIS's budget is not public, so the prior year is the comparison  |  Green = linked from Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. FY2025 VS FY2024, LINE BY LINE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fav. / Unfav.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Third straight year of growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large FY2022-FY2023 gifts rolling off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Program service revenue (school contracts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract revenue down for a second year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expenses by function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fastest-growing cost line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expenses by type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel (salaries, benefits, payroll tax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See the volume / rate split below</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All other expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total expenses less personnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: lines add up (revenue and expenses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fav. / Unfav. uses the standard convention: higher revenue or lower cost is favorable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. PERSONNEL COST: VOLUME VS RATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employees (Part I line 5, W-3 count)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel cost per employee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volume effect: added staff at FY2024 cost per person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(change in employees) x (FY2024 cost per employee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate effect: change in cost per person, at FY2025 headcount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(change in cost per employee) x (FY2025 employees)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total personnel change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: volume + rate = actual change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caveat: the W-3 count includes everyone paid during the calendar year, so turnover and part-time staff inflate it. That can overstate both the volume and the rate effects; full-time equivalents are not reported.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. DEFICIT BRIDGE: FY2024 SURPLUS TO FY2025 DEFICIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ impact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helps bottom line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hurts bottom line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY2024 surplus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel: more staff (volume)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel: lower cost per person (rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY2025 surplus / (deficit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: bridge ends at the FY2025 actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. WHAT DROVE THE CHANGE</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tab 3 - Forecast FY2026-FY2028  |  FY2025 = actual from the Form 990  |  Green = linked from another tab, black = calculated here</t>
   </si>
   <si>
@@ -789,9 +919,6 @@
   </si>
   <si>
     <t xml:space="preserve">FY2025 base grown at the government growth rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Program service revenue (school contracts)</t>
   </si>
   <si>
     <t xml:space="preserve">FY2025 actual grown at the program revenue growth rate</t>
@@ -1089,7 +1216,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.0,,\M"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0,,\M;&quot;($&quot;#,##0.0,,&quot;M)&quot;"/>
@@ -1104,6 +1231,7 @@
     <numFmt numFmtId="175" formatCode="#,##0"/>
     <numFmt numFmtId="176" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="177" formatCode="\$0.00"/>
+    <numFmt numFmtId="178" formatCode="\+#,##0;\-#,##0;\-"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -1370,7 +1498,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="79">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1563,6 +1691,18 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="175" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="176" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1701,8 +1841,8 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBEB9"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF8C8B87"/>
-      <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFF2F5FA"/>
@@ -2051,11 +2191,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="26896914"/>
-        <c:axId val="93646060"/>
+        <c:axId val="71845202"/>
+        <c:axId val="31155468"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="26896914"/>
+        <c:axId val="71845202"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2087,7 +2227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93646060"/>
+        <c:crossAx val="31155468"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2095,7 +2235,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93646060"/>
+        <c:axId val="31155468"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2134,7 +2274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26896914"/>
+        <c:crossAx val="71845202"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2485,11 +2625,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="28622519"/>
-        <c:axId val="55827632"/>
+        <c:axId val="4503622"/>
+        <c:axId val="75052577"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="28622519"/>
+        <c:axId val="4503622"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2521,7 +2661,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55827632"/>
+        <c:crossAx val="75052577"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2529,7 +2669,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55827632"/>
+        <c:axId val="75052577"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2602,7 +2742,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28622519"/>
+        <c:crossAx val="4503622"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3097,11 +3237,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="62880517"/>
-        <c:axId val="71035535"/>
+        <c:axId val="5256341"/>
+        <c:axId val="92481409"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="62880517"/>
+        <c:axId val="5256341"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3133,7 +3273,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71035535"/>
+        <c:crossAx val="92481409"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3141,7 +3281,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71035535"/>
+        <c:axId val="92481409"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3181,7 +3321,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62880517"/>
+        <c:crossAx val="5256341"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3577,11 +3717,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="89976692"/>
-        <c:axId val="15614599"/>
+        <c:axId val="27371469"/>
+        <c:axId val="62799528"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="89976692"/>
+        <c:axId val="27371469"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3613,7 +3753,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15614599"/>
+        <c:crossAx val="62799528"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3621,7 +3761,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15614599"/>
+        <c:axId val="62799528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3660,7 +3800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89976692"/>
+        <c:crossAx val="27371469"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3860,11 +4000,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="91644334"/>
-        <c:axId val="26995280"/>
+        <c:axId val="13384677"/>
+        <c:axId val="64568780"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91644334"/>
+        <c:axId val="13384677"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3896,7 +4036,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26995280"/>
+        <c:crossAx val="64568780"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3904,7 +4044,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26995280"/>
+        <c:axId val="64568780"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3943,7 +4083,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91644334"/>
+        <c:crossAx val="13384677"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3954,6 +4094,407 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1100" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="0b0b0b"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1100" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="0b0b0b"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>What moved the bottom line, FY2024 to FY2025</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Helps bottom line"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Helps bottom line</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2a78d6"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Variance!$A$40:$A$46</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Government grants</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Non-government contributions</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Program service revenue</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Investment &amp; other revenue</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Personnel: more staff (volume)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Personnel: lower cost per person (rate)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>All other expenses</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Variance!$D$40:$D$46</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>408865</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>873718.76744186</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>26779</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Hurts bottom line"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Hurts bottom line</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="eb6834"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Variance!$A$40:$A$46</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>Government grants</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Non-government contributions</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Program service revenue</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Investment &amp; other revenue</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Personnel: more staff (volume)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Personnel: lower cost per person (rate)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>All other expenses</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Variance!$E$40:$E$46</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-1541235</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-95750</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-36741</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-1199821.76744186</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="50"/>
+        <c:overlap val="100"/>
+        <c:axId val="9510455"/>
+        <c:axId val="90863277"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="9510455"/>
+        <c:scaling>
+          <c:orientation val="maxMin"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="52514e"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="90863277"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="90863277"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6480">
+              <a:solidFill>
+                <a:srgbClr val="e6e5e1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="\$#,##0.0,,\M;&quot;($&quot;#,##0.0,,&quot;M)&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="52514e"/>
+                </a:solidFill>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="9510455"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="900" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="52514e"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -4118,6 +4659,41 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>160920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>4680</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>172440</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="12100680" y="571680"/>
+        <a:ext cx="6119640" cy="3059640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -7336,6 +7912,777 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G54"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="47" t="n">
+        <f aca="false">Inputs!F13</f>
+        <v>580383</v>
+      </c>
+      <c r="C7" s="47" t="n">
+        <f aca="false">Inputs!G13</f>
+        <v>989248</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <f aca="false">C7-B7</f>
+        <v>408865</v>
+      </c>
+      <c r="E7" s="41" t="n">
+        <f aca="false">IF(B7=0,"n/a",(C7-B7)/ABS(B7))</f>
+        <v>0.704474459107176</v>
+      </c>
+      <c r="F7" s="19" t="str">
+        <f aca="false">IF(D7&gt;=0,"Favorable","Unfavorable")</f>
+        <v>Favorable</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="47" t="n">
+        <f aca="false">Inputs!F15</f>
+        <v>6745098</v>
+      </c>
+      <c r="C8" s="47" t="n">
+        <f aca="false">Inputs!G15</f>
+        <v>5203863</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <f aca="false">C8-B8</f>
+        <v>-1541235</v>
+      </c>
+      <c r="E8" s="41" t="n">
+        <f aca="false">IF(B8=0,"n/a",(C8-B8)/ABS(B8))</f>
+        <v>-0.228497050747076</v>
+      </c>
+      <c r="F8" s="19" t="str">
+        <f aca="false">IF(D8&gt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="B9" s="47" t="n">
+        <f aca="false">Inputs!F16</f>
+        <v>655750</v>
+      </c>
+      <c r="C9" s="47" t="n">
+        <f aca="false">Inputs!G16</f>
+        <v>560000</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <f aca="false">C9-B9</f>
+        <v>-95750</v>
+      </c>
+      <c r="E9" s="41" t="n">
+        <f aca="false">IF(B9=0,"n/a",(C9-B9)/ABS(B9))</f>
+        <v>-0.146016012199771</v>
+      </c>
+      <c r="F9" s="19" t="str">
+        <f aca="false">IF(D9&gt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="47" t="n">
+        <f aca="false">Inputs!F18</f>
+        <v>247695</v>
+      </c>
+      <c r="C10" s="47" t="n">
+        <f aca="false">Inputs!G18</f>
+        <v>210954</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <f aca="false">C10-B10</f>
+        <v>-36741</v>
+      </c>
+      <c r="E10" s="41" t="n">
+        <f aca="false">IF(B10=0,"n/a",(C10-B10)/ABS(B10))</f>
+        <v>-0.148331617513474</v>
+      </c>
+      <c r="F10" s="19" t="str">
+        <f aca="false">IF(D10&gt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="44" t="n">
+        <f aca="false">Inputs!F17</f>
+        <v>8228926</v>
+      </c>
+      <c r="C11" s="44" t="n">
+        <f aca="false">Inputs!G17</f>
+        <v>6964065</v>
+      </c>
+      <c r="D11" s="28" t="n">
+        <f aca="false">C11-B11</f>
+        <v>-1264861</v>
+      </c>
+      <c r="E11" s="42" t="n">
+        <f aca="false">IF(B11=0,"n/a",(C11-B11)/ABS(B11))</f>
+        <v>-0.153709123158964</v>
+      </c>
+      <c r="F11" s="19" t="str">
+        <f aca="false">IF(D11&gt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="47" t="n">
+        <f aca="false">Inputs!F21</f>
+        <v>5609813</v>
+      </c>
+      <c r="C14" s="47" t="n">
+        <f aca="false">Inputs!G21</f>
+        <v>5710185</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <f aca="false">C14-B14</f>
+        <v>100372</v>
+      </c>
+      <c r="E14" s="41" t="n">
+        <f aca="false">IF(B14=0,"n/a",(C14-B14)/ABS(B14))</f>
+        <v>0.0178922185106705</v>
+      </c>
+      <c r="F14" s="19" t="str">
+        <f aca="false">IF(D14&lt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="47" t="n">
+        <f aca="false">Inputs!F22</f>
+        <v>819140</v>
+      </c>
+      <c r="C15" s="47" t="n">
+        <f aca="false">Inputs!G22</f>
+        <v>1027814</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <f aca="false">C15-B15</f>
+        <v>208674</v>
+      </c>
+      <c r="E15" s="41" t="n">
+        <f aca="false">IF(B15=0,"n/a",(C15-B15)/ABS(B15))</f>
+        <v>0.254747662182289</v>
+      </c>
+      <c r="F15" s="19" t="str">
+        <f aca="false">IF(D15&lt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="47" t="n">
+        <f aca="false">Inputs!F23</f>
+        <v>1345742</v>
+      </c>
+      <c r="C16" s="47" t="n">
+        <f aca="false">Inputs!G23</f>
+        <v>1336020</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <f aca="false">C16-B16</f>
+        <v>-9722</v>
+      </c>
+      <c r="E16" s="41" t="n">
+        <f aca="false">IF(B16=0,"n/a",(C16-B16)/ABS(B16))</f>
+        <v>-0.00722426735585276</v>
+      </c>
+      <c r="F16" s="19" t="str">
+        <f aca="false">IF(D16&lt;=0,"Favorable","Unfavorable")</f>
+        <v>Favorable</v>
+      </c>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="44" t="n">
+        <f aca="false">Inputs!F24</f>
+        <v>7774695</v>
+      </c>
+      <c r="C17" s="44" t="n">
+        <f aca="false">Inputs!G24</f>
+        <v>8074019</v>
+      </c>
+      <c r="D17" s="28" t="n">
+        <f aca="false">C17-B17</f>
+        <v>299324</v>
+      </c>
+      <c r="E17" s="42" t="n">
+        <f aca="false">IF(B17=0,"n/a",(C17-B17)/ABS(B17))</f>
+        <v>0.0384997739461162</v>
+      </c>
+      <c r="F17" s="19" t="str">
+        <f aca="false">IF(D17&lt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23" t="s">
+        <v>234</v>
+      </c>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="B19" s="47" t="n">
+        <f aca="false">Inputs!F25</f>
+        <v>6449042</v>
+      </c>
+      <c r="C19" s="47" t="n">
+        <f aca="false">Inputs!G25</f>
+        <v>6775145</v>
+      </c>
+      <c r="D19" s="27" t="n">
+        <f aca="false">C19-B19</f>
+        <v>326103</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <f aca="false">IF(B19=0,"n/a",(C19-B19)/ABS(B19))</f>
+        <v>0.0505661150912027</v>
+      </c>
+      <c r="F19" s="19" t="str">
+        <f aca="false">IF(D19&lt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="B20" s="27" t="n">
+        <f aca="false">B17-B19</f>
+        <v>1325653</v>
+      </c>
+      <c r="C20" s="27" t="n">
+        <f aca="false">C17-C19</f>
+        <v>1298874</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <f aca="false">C20-B20</f>
+        <v>-26779</v>
+      </c>
+      <c r="E20" s="41" t="n">
+        <f aca="false">IF(B20=0,"n/a",(C20-B20)/ABS(B20))</f>
+        <v>-0.0202006105670187</v>
+      </c>
+      <c r="F20" s="19" t="str">
+        <f aca="false">IF(D20&lt;=0,"Favorable","Unfavorable")</f>
+        <v>Favorable</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" s="44" t="n">
+        <f aca="false">Inputs!F26</f>
+        <v>454231</v>
+      </c>
+      <c r="C22" s="44" t="n">
+        <f aca="false">Inputs!G26</f>
+        <v>-1109954</v>
+      </c>
+      <c r="D22" s="28" t="n">
+        <f aca="false">C22-B22</f>
+        <v>-1564185</v>
+      </c>
+      <c r="E22" s="42" t="str">
+        <f aca="false">"n/a"</f>
+        <v>n/a</v>
+      </c>
+      <c r="F22" s="19" t="str">
+        <f aca="false">IF(D22&gt;=0,"Favorable","Unfavorable")</f>
+        <v>Unfavorable</v>
+      </c>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="D23" s="13" t="str">
+        <f aca="false">IF(AND(ABS(SUM(D7:D10)-D11)&lt;=1,ABS(SUM(D14:D16)-D17)&lt;=1,ABS(D19+D20-D17)&lt;=1),"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="B27" s="48" t="n">
+        <f aca="false">Inputs!F43</f>
+        <v>86</v>
+      </c>
+      <c r="C27" s="48" t="n">
+        <f aca="false">Inputs!G43</f>
+        <v>102</v>
+      </c>
+      <c r="D27" s="49" t="n">
+        <f aca="false">C27-B27</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="B28" s="47" t="n">
+        <f aca="false">Inputs!F25</f>
+        <v>6449042</v>
+      </c>
+      <c r="C28" s="47" t="n">
+        <f aca="false">Inputs!G25</f>
+        <v>6775145</v>
+      </c>
+      <c r="D28" s="27" t="n">
+        <f aca="false">C28-B28</f>
+        <v>326103</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="B29" s="27" t="n">
+        <f aca="false">B28/B27</f>
+        <v>74988.8604651163</v>
+      </c>
+      <c r="C29" s="27" t="n">
+        <f aca="false">C28/C27</f>
+        <v>66422.9901960784</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <f aca="false">C29-B29</f>
+        <v>-8565.87026903784</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="D31" s="28" t="n">
+        <f aca="false">(C27-B27)*B29</f>
+        <v>1199821.76744186</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D32" s="28" t="n">
+        <f aca="false">(C29-B29)*C27</f>
+        <v>-873718.76744186</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D33" s="28" t="n">
+        <f aca="false">D31+D32</f>
+        <v>326103.000000001</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="D34" s="13" t="str">
+        <f aca="false">IF(ABS(D33-D28)&lt;=1,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21" t="s">
+        <v>254</v>
+      </c>
+      <c r="B38" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="B39" s="28" t="n">
+        <f aca="false">B22</f>
+        <v>454231</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" s="27" t="n">
+        <f aca="false">D7</f>
+        <v>408865</v>
+      </c>
+      <c r="D40" s="50" t="n">
+        <f aca="false">MAX(0,B40)</f>
+        <v>408865</v>
+      </c>
+      <c r="E40" s="50" t="n">
+        <f aca="false">MIN(0,B40)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="27" t="n">
+        <f aca="false">D8</f>
+        <v>-1541235</v>
+      </c>
+      <c r="D41" s="50" t="n">
+        <f aca="false">MAX(0,B41)</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="50" t="n">
+        <f aca="false">MIN(0,B41)</f>
+        <v>-1541235</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42" s="27" t="n">
+        <f aca="false">D9</f>
+        <v>-95750</v>
+      </c>
+      <c r="D42" s="50" t="n">
+        <f aca="false">MAX(0,B42)</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="50" t="n">
+        <f aca="false">MIN(0,B42)</f>
+        <v>-95750</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B43" s="27" t="n">
+        <f aca="false">D10</f>
+        <v>-36741</v>
+      </c>
+      <c r="D43" s="50" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="50" t="n">
+        <f aca="false">MIN(0,B43)</f>
+        <v>-36741</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="B44" s="27" t="n">
+        <f aca="false">-D31</f>
+        <v>-1199821.76744186</v>
+      </c>
+      <c r="D44" s="50" t="n">
+        <f aca="false">MAX(0,B44)</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="50" t="n">
+        <f aca="false">MIN(0,B44)</f>
+        <v>-1199821.76744186</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B45" s="27" t="n">
+        <f aca="false">-D32</f>
+        <v>873718.76744186</v>
+      </c>
+      <c r="D45" s="50" t="n">
+        <f aca="false">MAX(0,B45)</f>
+        <v>873718.76744186</v>
+      </c>
+      <c r="E45" s="50" t="n">
+        <f aca="false">MIN(0,B45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="B46" s="27" t="n">
+        <f aca="false">-D20</f>
+        <v>26779</v>
+      </c>
+      <c r="D46" s="50" t="n">
+        <f aca="false">MAX(0,B46)</f>
+        <v>26779</v>
+      </c>
+      <c r="E46" s="50" t="n">
+        <f aca="false">MIN(0,B46)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="B47" s="28" t="n">
+        <f aca="false">SUM(B39:B46)</f>
+        <v>-1109954</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="B48" s="13" t="str">
+        <f aca="false">IF(ABS(B47-C22)&lt;=1,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="B50" s="11"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+      <c r="G50" s="11"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="str">
+        <f aca="false">"Revenue fell "&amp;TEXT(-E11,"0%")&amp;" ("&amp;TEXT(ABS(D11)/1000000,"$0.0")&amp;"M"&amp;"), driven by non-government contributions (down "&amp;TEXT(ABS(D8)/1000000,"$0.0")&amp;"M"&amp;") as the large FY2022-FY2023 gifts rolled off. Government grants partly offset this (up "&amp;TEXT(ABS(D7)/1000000,"$0.0")&amp;"M"&amp;")."</f>
+        <v>Revenue fell 15% ($1.3M), driven by non-government contributions (down $1.5M) as the large FY2022-FY2023 gifts rolled off. Government grants partly offset this (up $0.4M).</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="str">
+        <f aca="false">"Expenses rose only "&amp;TEXT(E17,"0.0%")&amp;". Personnel was up "&amp;TEXT(ABS(D28)/1000000,"$0.0")&amp;"M"&amp;": "&amp;D27&amp;" more staff added about "&amp;TEXT(ABS(D31)/1000000,"$0.0")&amp;"M"&amp;", offset by about "&amp;TEXT(ABS(D32)/1000000,"$0.0")&amp;"M"&amp;" from a lower cost per employee."</f>
+        <v>Expenses rose only 3.8%. Personnel was up $0.3M: 16 more staff added about $1.2M, offset by about $0.9M from a lower cost per employee.</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="str">
+        <f aca="false">"Management &amp; general grew "&amp;TEXT(E15,"0%")&amp;", the fastest of any cost line, while program services grew "&amp;TEXT(E14,"0.0%")&amp;"."</f>
+        <v>Management &amp; general grew 25%, the fastest of any cost line, while program services grew 1.8%.</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="str">
+        <f aca="false">"Net result: a "&amp;TEXT(ABS(C22-B22)/1000000,"$0.0")&amp;"M"&amp;" swing, from a "&amp;TEXT(ABS(B22)/1000000,"$0.0")&amp;"M"&amp;" surplus to a "&amp;TEXT(ABS(C22)/1000000,"$0.0")&amp;"M"&amp;" deficit. The FY2025 deficit is mainly a revenue problem (gifts rolling off), not a cost blow-out."</f>
+        <v>Net result: a $1.6M swing, from a $0.5M surplus to a $1.1M deficit. The FY2025 deficit is mainly a revenue problem (gifts rolling off), not a cost blow-out.</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -7351,12 +8698,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>221</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>222</v>
+        <v>265</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -7375,7 +8722,7 @@
       <c r="D5" s="32"/>
       <c r="E5" s="32"/>
       <c r="F5" s="31" t="s">
-        <v>223</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7387,19 +8734,19 @@
         <v>5203863</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>224</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="48" t="n">
+      <c r="C7" s="51" t="n">
         <f aca="false">Scenarios!H12</f>
         <v>0.03</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>225</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7411,31 +8758,31 @@
         <v>989248</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>226</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C9" s="48" t="n">
+      <c r="C9" s="51" t="n">
         <f aca="false">Scenarios!H14</f>
         <v>0</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>227</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="C10" s="49" t="n">
+        <v>271</v>
+      </c>
+      <c r="C10" s="52" t="n">
         <f aca="false">Scenarios!H15</f>
         <v>1</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>229</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7447,91 +8794,91 @@
         <v>5000000</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>230</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>231</v>
-      </c>
-      <c r="C12" s="49" t="n">
+        <v>274</v>
+      </c>
+      <c r="C12" s="52" t="n">
         <f aca="false">Scenarios!H17</f>
         <v>4</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>232</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C13" s="49" t="n">
+      <c r="C13" s="52" t="n">
         <f aca="false">Scenarios!H18</f>
         <v>2023</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>233</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="51" t="n">
         <f aca="false">Scenarios!H19</f>
         <v>0</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>234</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>235</v>
+        <v>278</v>
       </c>
       <c r="C15" s="47" t="n">
         <f aca="false">Scenarios!H20</f>
         <v>210954</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>236</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="51" t="n">
         <f aca="false">Scenarios!H21</f>
         <v>0.06</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>237</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="C17" s="50" t="n">
+        <v>281</v>
+      </c>
+      <c r="C17" s="53" t="n">
         <f aca="false">Scenarios!H22</f>
         <v>3</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>239</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="C18" s="49" t="n">
+        <v>283</v>
+      </c>
+      <c r="C18" s="52" t="n">
         <f aca="false">Scenarios!H23</f>
         <v>1</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>241</v>
+        <v>284</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7543,24 +8890,24 @@
         <v>1237082</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>242</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="52" t="n">
         <f aca="false">Scenarios!H25</f>
         <v>3</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>243</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>244</v>
+        <v>287</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -7572,38 +8919,38 @@
       <c r="A23" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="51" t="s">
-        <v>245</v>
+      <c r="B23" s="54" t="s">
+        <v>288</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>246</v>
+        <v>289</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>247</v>
+        <v>290</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>248</v>
+        <v>291</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>249</v>
+        <v>292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B24" s="52" t="n">
+        <v>293</v>
+      </c>
+      <c r="B24" s="55" t="n">
         <v>2025</v>
       </c>
-      <c r="C24" s="53" t="n">
+      <c r="C24" s="56" t="n">
         <f aca="false">B24+1</f>
         <v>2026</v>
       </c>
-      <c r="D24" s="53" t="n">
+      <c r="D24" s="56" t="n">
         <f aca="false">C24+1</f>
         <v>2027</v>
       </c>
-      <c r="E24" s="53" t="n">
+      <c r="E24" s="56" t="n">
         <f aca="false">D24+1</f>
         <v>2028</v>
       </c>
@@ -7620,9 +8967,9 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="B26" s="54" t="n">
+        <v>294</v>
+      </c>
+      <c r="B26" s="57" t="n">
         <f aca="false">Inputs!G14-Inputs!G13</f>
         <v>5203863</v>
       </c>
@@ -7639,14 +8986,14 @@
         <v>5686401.604401</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>252</v>
+        <v>295</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="54" t="n">
+      <c r="B27" s="57" t="n">
         <f aca="false">Inputs!G13</f>
         <v>989248</v>
       </c>
@@ -7663,14 +9010,14 @@
         <v>989248</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>253</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="B28" s="54" t="n">
+        <v>230</v>
+      </c>
+      <c r="B28" s="57" t="n">
         <f aca="false">Inputs!G16</f>
         <v>560000</v>
       </c>
@@ -7687,14 +9034,14 @@
         <v>560000</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>255</v>
+        <v>297</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B29" s="54" t="n">
+      <c r="B29" s="57" t="n">
         <f aca="false">Inputs!G18</f>
         <v>210954</v>
       </c>
@@ -7711,14 +9058,14 @@
         <v>210954</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>256</v>
+        <v>298</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>257</v>
-      </c>
-      <c r="B30" s="55" t="n">
+        <v>299</v>
+      </c>
+      <c r="B30" s="58" t="n">
         <f aca="false">SUM(B26:B29)</f>
         <v>6964065</v>
       </c>
@@ -7735,14 +9082,14 @@
         <v>7446603.604401</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>258</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="B31" s="56" t="n">
+        <v>301</v>
+      </c>
+      <c r="B31" s="59" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="27" t="n">
@@ -7758,14 +9105,14 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>260</v>
+        <v>302</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="B32" s="55" t="n">
+        <v>303</v>
+      </c>
+      <c r="B32" s="58" t="n">
         <f aca="false">B30+B31</f>
         <v>6964065</v>
       </c>
@@ -7782,7 +9129,7 @@
         <v>7446603.604401</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7799,7 +9146,7 @@
       <c r="A34" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="57" t="n">
+      <c r="B34" s="60" t="n">
         <f aca="false">Inputs!G24</f>
         <v>8074019</v>
       </c>
@@ -7816,12 +9163,12 @@
         <v>9616285.813304</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>263</v>
+        <v>305</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23" t="s">
-        <v>264</v>
+        <v>306</v>
       </c>
       <c r="B35" s="24"/>
       <c r="C35" s="24"/>
@@ -7831,9 +9178,9 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>265</v>
-      </c>
-      <c r="B36" s="55" t="n">
+        <v>307</v>
+      </c>
+      <c r="B36" s="58" t="n">
         <f aca="false">B30-B34</f>
         <v>-1109954</v>
       </c>
@@ -7850,14 +9197,14 @@
         <v>-2169682.208903</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>266</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>267</v>
-      </c>
-      <c r="B37" s="56" t="n">
+        <v>309</v>
+      </c>
+      <c r="B37" s="59" t="n">
         <f aca="false">B32-B34</f>
         <v>-1109954</v>
       </c>
@@ -7874,14 +9221,14 @@
         <v>-2169682.208903</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>268</v>
+        <v>310</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="B38" s="58" t="n">
+        <v>311</v>
+      </c>
+      <c r="B38" s="61" t="n">
         <f aca="false">B36/B30</f>
         <v>-0.159383061473435</v>
       </c>
@@ -7898,12 +9245,12 @@
         <v>-0.291365342398607</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>270</v>
+        <v>312</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23" t="s">
-        <v>271</v>
+        <v>313</v>
       </c>
       <c r="B39" s="24"/>
       <c r="C39" s="24"/>
@@ -7913,9 +9260,9 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>272</v>
-      </c>
-      <c r="B40" s="59"/>
+        <v>314</v>
+      </c>
+      <c r="B40" s="62"/>
       <c r="C40" s="27" t="n">
         <f aca="false">B43</f>
         <v>6396696</v>
@@ -7929,14 +9276,14 @@
         <v>7927876.59163333</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>273</v>
+        <v>315</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>274</v>
-      </c>
-      <c r="B41" s="59"/>
+        <v>316</v>
+      </c>
+      <c r="B41" s="62"/>
       <c r="C41" s="27" t="n">
         <f aca="false">SUMPRODUCT($C$31:C31*((C$24-$C$24:C$24)&lt;$C$12))/$C$12</f>
         <v>0</v>
@@ -7950,14 +9297,14 @@
         <v>1250000</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>275</v>
+        <v>317</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>276</v>
-      </c>
-      <c r="B42" s="59"/>
+        <v>318</v>
+      </c>
+      <c r="B42" s="62"/>
       <c r="C42" s="27" t="n">
         <f aca="false">IF(AND($C$18=1,(C$24-$B$24)&lt;=$C$20),MAX(0,Inputs!$G$37-$C$19)/$C$20,0)</f>
         <v>1755223.66666667</v>
@@ -7971,14 +9318,14 @@
         <v>1755223.66666667</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>277</v>
+        <v>319</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="B43" s="57" t="n">
+        <v>320</v>
+      </c>
+      <c r="B43" s="60" t="n">
         <f aca="false">Inputs!G36</f>
         <v>6396696</v>
       </c>
@@ -7995,14 +9342,14 @@
         <v>8763418.049397</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>279</v>
+        <v>321</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="B44" s="54" t="n">
+        <v>322</v>
+      </c>
+      <c r="B44" s="57" t="n">
         <f aca="false">Inputs!G37</f>
         <v>6502753</v>
       </c>
@@ -8019,14 +9366,14 @@
         <v>3737082</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>281</v>
+        <v>323</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="B45" s="54" t="n">
+        <v>324</v>
+      </c>
+      <c r="B45" s="57" t="n">
         <f aca="false">Inputs!G38</f>
         <v>12899449</v>
       </c>
@@ -8043,14 +9390,14 @@
         <v>12500500.049397</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>283</v>
+        <v>325</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="B46" s="56" t="n">
+      <c r="B46" s="59" t="n">
         <f aca="false">B34/12</f>
         <v>672834.916666667</v>
       </c>
@@ -8074,31 +9421,31 @@
       <c r="A47" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="60" t="n">
+      <c r="B47" s="63" t="n">
         <f aca="false">B43/B46</f>
         <v>9.5070809221529</v>
       </c>
-      <c r="C47" s="61" t="n">
+      <c r="C47" s="64" t="n">
         <f aca="false">C43/C46</f>
         <v>9.41333881120348</v>
       </c>
-      <c r="D47" s="61" t="n">
+      <c r="D47" s="64" t="n">
         <f aca="false">D43/D46</f>
         <v>10.4866465289604</v>
       </c>
-      <c r="E47" s="61" t="n">
+      <c r="E47" s="64" t="n">
         <f aca="false">E43/E46</f>
         <v>10.9357207797708</v>
       </c>
       <c r="F47" s="26" t="s">
-        <v>284</v>
+        <v>326</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="B48" s="62" t="n">
+        <v>327</v>
+      </c>
+      <c r="B48" s="65" t="n">
         <f aca="false">B47-$C$17</f>
         <v>6.5070809221529</v>
       </c>
@@ -8115,14 +9462,14 @@
         <v>7.93572077977083</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>286</v>
+        <v>328</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="s">
-        <v>287</v>
-      </c>
-      <c r="B49" s="63" t="str">
+        <v>329</v>
+      </c>
+      <c r="B49" s="66" t="str">
         <f aca="false">IF(B47&lt;$C$17,"BELOW FLOOR","OK")</f>
         <v>OK</v>
       </c>
@@ -8142,7 +9489,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
-        <v>288</v>
+        <v>330</v>
       </c>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
@@ -8152,7 +9499,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>289</v>
+        <v>331</v>
       </c>
       <c r="C52" s="28" t="n">
         <f aca="false">E43</f>
@@ -8161,25 +9508,25 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="C53" s="61" t="n">
+        <v>332</v>
+      </c>
+      <c r="C53" s="64" t="n">
         <f aca="false">E47</f>
         <v>10.9357207797708</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="C54" s="64" t="str">
+        <v>333</v>
+      </c>
+      <c r="C54" s="67" t="str">
         <f aca="false">IFERROR(INDEX(C23:E23,MATCH("BELOW FLOOR",C49:E49,0)),"Not within FY2026-FY2028")</f>
         <v>Not within FY2026-FY2028</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>292</v>
+        <v>334</v>
       </c>
       <c r="C55" s="28" t="n">
         <f aca="false">SUM(C36:E36)</f>
@@ -8188,7 +9535,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>293</v>
+        <v>335</v>
       </c>
       <c r="C56" s="28" t="n">
         <f aca="false">-AVERAGE(C36:E36)</f>
@@ -8197,34 +9544,34 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>294</v>
-      </c>
-      <c r="C57" s="65" t="n">
+        <v>336</v>
+      </c>
+      <c r="C57" s="68" t="n">
         <f aca="false">IF(E36&lt;0,E43/-E36,"n/a")</f>
         <v>4.03903300374473</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>295</v>
-      </c>
-      <c r="C58" s="64" t="str">
+        <v>337</v>
+      </c>
+      <c r="C58" s="67" t="str">
         <f aca="false">IF(ABS(B32-Inputs!G17)&lt;=1,"OK","CHECK")</f>
         <v>OK</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="C59" s="64" t="str">
+        <v>338</v>
+      </c>
+      <c r="C59" s="67" t="str">
         <f aca="false">IF(ABS(E45-B45-SUM(C37:E37))&lt;=1,"OK","CHECK")</f>
         <v>OK</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>297</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -8238,7 +9585,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -8259,12 +9606,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>298</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>299</v>
+        <v>341</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -8277,27 +9624,27 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>300</v>
-      </c>
-      <c r="C5" s="66" t="s">
-        <v>301</v>
+        <v>342</v>
+      </c>
+      <c r="C5" s="69" t="s">
+        <v>343</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>302</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="C6" s="53" t="n">
+        <v>345</v>
+      </c>
+      <c r="C6" s="56" t="n">
         <f aca="false">MATCH(C5,C9:G9,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>304</v>
+        <v>346</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -8314,45 +9661,45 @@
       </c>
       <c r="B9" s="32"/>
       <c r="C9" s="22" t="s">
-        <v>301</v>
+        <v>343</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>305</v>
+        <v>347</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>306</v>
+        <v>348</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>307</v>
+        <v>349</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>308</v>
-      </c>
-      <c r="H9" s="67" t="s">
-        <v>309</v>
+        <v>350</v>
+      </c>
+      <c r="H9" s="70" t="s">
+        <v>351</v>
       </c>
       <c r="I9" s="31" t="s">
-        <v>310</v>
+        <v>352</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C10" s="68" t="s">
-        <v>312</v>
-      </c>
-      <c r="D10" s="68" t="s">
-        <v>313</v>
-      </c>
-      <c r="E10" s="68" t="s">
-        <v>314</v>
-      </c>
-      <c r="F10" s="68" t="s">
-        <v>315</v>
-      </c>
-      <c r="G10" s="68" t="s">
-        <v>316</v>
+        <v>353</v>
+      </c>
+      <c r="C10" s="71" t="s">
+        <v>354</v>
+      </c>
+      <c r="D10" s="71" t="s">
+        <v>355</v>
+      </c>
+      <c r="E10" s="71" t="s">
+        <v>356</v>
+      </c>
+      <c r="F10" s="71" t="s">
+        <v>357</v>
+      </c>
+      <c r="G10" s="71" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8379,7 +9726,7 @@
         <f aca="false">$C11</f>
         <v>5203863</v>
       </c>
-      <c r="H11" s="69" t="n">
+      <c r="H11" s="72" t="n">
         <f aca="false">INDEX(C11:G11,$C$6)</f>
         <v>5203863</v>
       </c>
@@ -8388,27 +9735,27 @@
       <c r="A12" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="C12" s="48" t="n">
+      <c r="C12" s="51" t="n">
         <f aca="false">Inputs!C48</f>
         <v>0.03</v>
       </c>
-      <c r="D12" s="48" t="n">
+      <c r="D12" s="51" t="n">
         <f aca="false">$C12</f>
         <v>0.03</v>
       </c>
-      <c r="E12" s="48" t="n">
+      <c r="E12" s="51" t="n">
         <f aca="false">$C12</f>
         <v>0.03</v>
       </c>
-      <c r="F12" s="48" t="n">
+      <c r="F12" s="51" t="n">
         <f aca="false">$C12</f>
         <v>0.03</v>
       </c>
-      <c r="G12" s="48" t="n">
+      <c r="G12" s="51" t="n">
         <f aca="false">$C12</f>
         <v>0.03</v>
       </c>
-      <c r="H12" s="70" t="n">
+      <c r="H12" s="73" t="n">
         <f aca="false">INDEX(C12:G12,$C$6)</f>
         <v>0.03</v>
       </c>
@@ -8437,71 +9784,71 @@
         <f aca="false">$C13*(1-$C$27)</f>
         <v>494624</v>
       </c>
-      <c r="H13" s="69" t="n">
+      <c r="H13" s="72" t="n">
         <f aca="false">INDEX(C13:G13,$C$6)</f>
         <v>989248</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>317</v>
+        <v>359</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="51" t="n">
         <f aca="false">Inputs!C50</f>
         <v>0</v>
       </c>
-      <c r="D14" s="48" t="n">
+      <c r="D14" s="51" t="n">
         <f aca="false">$C14</f>
         <v>0</v>
       </c>
-      <c r="E14" s="48" t="n">
+      <c r="E14" s="51" t="n">
         <f aca="false">$C14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="48" t="n">
+      <c r="F14" s="51" t="n">
         <f aca="false">$C14</f>
         <v>0</v>
       </c>
-      <c r="G14" s="48" t="n">
+      <c r="G14" s="51" t="n">
         <f aca="false">$C14</f>
         <v>0</v>
       </c>
-      <c r="H14" s="70" t="n">
+      <c r="H14" s="73" t="n">
         <f aca="false">INDEX(C14:G14,$C$6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="C15" s="49" t="n">
+        <v>271</v>
+      </c>
+      <c r="C15" s="52" t="n">
         <f aca="false">Inputs!C51</f>
         <v>1</v>
       </c>
-      <c r="D15" s="71" t="n">
+      <c r="D15" s="74" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="49" t="n">
+      <c r="E15" s="52" t="n">
         <f aca="false">$C15</f>
         <v>1</v>
       </c>
-      <c r="F15" s="49" t="n">
+      <c r="F15" s="52" t="n">
         <f aca="false">$C15</f>
         <v>1</v>
       </c>
-      <c r="G15" s="71" t="n">
+      <c r="G15" s="74" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="72" t="n">
+      <c r="H15" s="75" t="n">
         <f aca="false">INDEX(C15:G15,$C$6)</f>
         <v>1</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>318</v>
+        <v>360</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8528,36 +9875,36 @@
         <f aca="false">$C16</f>
         <v>5000000</v>
       </c>
-      <c r="H16" s="69" t="n">
+      <c r="H16" s="72" t="n">
         <f aca="false">INDEX(C16:G16,$C$6)</f>
         <v>5000000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>319</v>
-      </c>
-      <c r="C17" s="49" t="n">
+        <v>361</v>
+      </c>
+      <c r="C17" s="52" t="n">
         <f aca="false">Inputs!C53</f>
         <v>4</v>
       </c>
-      <c r="D17" s="49" t="n">
+      <c r="D17" s="52" t="n">
         <f aca="false">$C17</f>
         <v>4</v>
       </c>
-      <c r="E17" s="49" t="n">
+      <c r="E17" s="52" t="n">
         <f aca="false">$C17</f>
         <v>4</v>
       </c>
-      <c r="F17" s="49" t="n">
+      <c r="F17" s="52" t="n">
         <f aca="false">$C17</f>
         <v>4</v>
       </c>
-      <c r="G17" s="49" t="n">
+      <c r="G17" s="52" t="n">
         <f aca="false">$C17</f>
         <v>4</v>
       </c>
-      <c r="H17" s="72" t="n">
+      <c r="H17" s="75" t="n">
         <f aca="false">INDEX(C17:G17,$C$6)</f>
         <v>4</v>
       </c>
@@ -8566,27 +9913,27 @@
       <c r="A18" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="49" t="n">
+      <c r="C18" s="52" t="n">
         <f aca="false">Inputs!C54</f>
         <v>2023</v>
       </c>
-      <c r="D18" s="49" t="n">
+      <c r="D18" s="52" t="n">
         <f aca="false">$C18</f>
         <v>2023</v>
       </c>
-      <c r="E18" s="49" t="n">
+      <c r="E18" s="52" t="n">
         <f aca="false">$C18</f>
         <v>2023</v>
       </c>
-      <c r="F18" s="49" t="n">
+      <c r="F18" s="52" t="n">
         <f aca="false">$C18</f>
         <v>2023</v>
       </c>
-      <c r="G18" s="49" t="n">
+      <c r="G18" s="52" t="n">
         <f aca="false">$C18</f>
         <v>2023</v>
       </c>
-      <c r="H18" s="72" t="n">
+      <c r="H18" s="75" t="n">
         <f aca="false">INDEX(C18:G18,$C$6)</f>
         <v>2023</v>
       </c>
@@ -8595,34 +9942,34 @@
       <c r="A19" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="51" t="n">
         <f aca="false">Inputs!C55</f>
         <v>0</v>
       </c>
-      <c r="D19" s="48" t="n">
+      <c r="D19" s="51" t="n">
         <f aca="false">$C19</f>
         <v>0</v>
       </c>
-      <c r="E19" s="48" t="n">
+      <c r="E19" s="51" t="n">
         <f aca="false">$C19</f>
         <v>0</v>
       </c>
-      <c r="F19" s="48" t="n">
+      <c r="F19" s="51" t="n">
         <f aca="false">$C19</f>
         <v>0</v>
       </c>
-      <c r="G19" s="48" t="n">
+      <c r="G19" s="51" t="n">
         <f aca="false">$C19</f>
         <v>0</v>
       </c>
-      <c r="H19" s="70" t="n">
+      <c r="H19" s="73" t="n">
         <f aca="false">INDEX(C19:G19,$C$6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>235</v>
+        <v>278</v>
       </c>
       <c r="C20" s="47" t="n">
         <f aca="false">Inputs!C56</f>
@@ -8644,7 +9991,7 @@
         <f aca="false">$C20</f>
         <v>210954</v>
       </c>
-      <c r="H20" s="69" t="n">
+      <c r="H20" s="72" t="n">
         <f aca="false">INDEX(C20:G20,$C$6)</f>
         <v>210954</v>
       </c>
@@ -8653,92 +10000,92 @@
       <c r="A21" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="C21" s="48" t="n">
+      <c r="C21" s="51" t="n">
         <f aca="false">Inputs!C57</f>
         <v>0.06</v>
       </c>
-      <c r="D21" s="48" t="n">
+      <c r="D21" s="51" t="n">
         <f aca="false">$C21</f>
         <v>0.06</v>
       </c>
-      <c r="E21" s="48" t="n">
+      <c r="E21" s="51" t="n">
         <f aca="false">$C21</f>
         <v>0.06</v>
       </c>
-      <c r="F21" s="73" t="n">
+      <c r="F21" s="76" t="n">
         <v>0.03</v>
       </c>
-      <c r="G21" s="48" t="n">
+      <c r="G21" s="51" t="n">
         <f aca="false">$C21</f>
         <v>0.06</v>
       </c>
-      <c r="H21" s="70" t="n">
+      <c r="H21" s="73" t="n">
         <f aca="false">INDEX(C21:G21,$C$6)</f>
         <v>0.06</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>320</v>
+        <v>362</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="C22" s="50" t="n">
+        <v>281</v>
+      </c>
+      <c r="C22" s="53" t="n">
         <f aca="false">Inputs!C59</f>
         <v>3</v>
       </c>
-      <c r="D22" s="50" t="n">
+      <c r="D22" s="53" t="n">
         <f aca="false">$C22</f>
         <v>3</v>
       </c>
-      <c r="E22" s="50" t="n">
+      <c r="E22" s="53" t="n">
         <f aca="false">$C22</f>
         <v>3</v>
       </c>
-      <c r="F22" s="50" t="n">
+      <c r="F22" s="53" t="n">
         <f aca="false">$C22</f>
         <v>3</v>
       </c>
-      <c r="G22" s="50" t="n">
+      <c r="G22" s="53" t="n">
         <f aca="false">$C22</f>
         <v>3</v>
       </c>
-      <c r="H22" s="74" t="n">
+      <c r="H22" s="77" t="n">
         <f aca="false">INDEX(C22:G22,$C$6)</f>
         <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="C23" s="49" t="n">
+        <v>283</v>
+      </c>
+      <c r="C23" s="52" t="n">
         <f aca="false">Inputs!C60</f>
         <v>1</v>
       </c>
-      <c r="D23" s="49" t="n">
+      <c r="D23" s="52" t="n">
         <f aca="false">$C23</f>
         <v>1</v>
       </c>
-      <c r="E23" s="49" t="n">
+      <c r="E23" s="52" t="n">
         <f aca="false">$C23</f>
         <v>1</v>
       </c>
-      <c r="F23" s="49" t="n">
+      <c r="F23" s="52" t="n">
         <f aca="false">$C23</f>
         <v>1</v>
       </c>
-      <c r="G23" s="49" t="n">
+      <c r="G23" s="52" t="n">
         <f aca="false">$C23</f>
         <v>1</v>
       </c>
-      <c r="H23" s="72" t="n">
+      <c r="H23" s="75" t="n">
         <f aca="false">INDEX(C23:G23,$C$6)</f>
         <v>1</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>321</v>
+        <v>363</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8765,7 +10112,7 @@
         <f aca="false">$C24</f>
         <v>1237082</v>
       </c>
-      <c r="H24" s="69" t="n">
+      <c r="H24" s="72" t="n">
         <f aca="false">INDEX(C24:G24,$C$6)</f>
         <v>1237082</v>
       </c>
@@ -8774,45 +10121,45 @@
       <c r="A25" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="C25" s="49" t="n">
+      <c r="C25" s="52" t="n">
         <f aca="false">Inputs!C62</f>
         <v>3</v>
       </c>
-      <c r="D25" s="49" t="n">
+      <c r="D25" s="52" t="n">
         <f aca="false">$C25</f>
         <v>3</v>
       </c>
-      <c r="E25" s="49" t="n">
+      <c r="E25" s="52" t="n">
         <f aca="false">$C25</f>
         <v>3</v>
       </c>
-      <c r="F25" s="49" t="n">
+      <c r="F25" s="52" t="n">
         <f aca="false">$C25</f>
         <v>3</v>
       </c>
-      <c r="G25" s="49" t="n">
+      <c r="G25" s="52" t="n">
         <f aca="false">$C25</f>
         <v>3</v>
       </c>
-      <c r="H25" s="72" t="n">
+      <c r="H25" s="75" t="n">
         <f aca="false">INDEX(C25:G25,$C$6)</f>
         <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="C27" s="73" t="n">
+        <v>364</v>
+      </c>
+      <c r="C27" s="76" t="n">
         <v>0.5</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>323</v>
+        <v>365</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>324</v>
+        <v>366</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -8850,12 +10197,12 @@
       </c>
       <c r="H30" s="32"/>
       <c r="I30" s="31" t="s">
-        <v>325</v>
+        <v>367</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>326</v>
+        <v>368</v>
       </c>
       <c r="C31" s="27" t="n">
         <f aca="false">E56</f>
@@ -8878,40 +10225,40 @@
         <v>4779546.049397</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>327</v>
+        <v>369</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="C32" s="61" t="n">
+        <v>370</v>
+      </c>
+      <c r="C32" s="64" t="n">
         <f aca="false">E57</f>
         <v>10.9357207797708</v>
       </c>
-      <c r="D32" s="61" t="n">
+      <c r="D32" s="64" t="n">
         <f aca="false">E68</f>
         <v>7.81601317306727</v>
       </c>
-      <c r="E32" s="61" t="n">
+      <c r="E32" s="64" t="n">
         <f aca="false">E79</f>
         <v>9.08402207346106</v>
       </c>
-      <c r="F32" s="61" t="n">
+      <c r="F32" s="64" t="n">
         <f aca="false">E90</f>
         <v>14.0167547980781</v>
       </c>
-      <c r="G32" s="61" t="n">
+      <c r="G32" s="64" t="n">
         <f aca="false">E101</f>
         <v>5.9643144667575</v>
       </c>
       <c r="I32" s="26" t="s">
-        <v>329</v>
+        <v>371</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>330</v>
+        <v>372</v>
       </c>
       <c r="C33" s="45" t="n">
         <f aca="false">MIN(C57:E57)</f>
@@ -8937,7 +10284,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>291</v>
+        <v>333</v>
       </c>
       <c r="C34" s="19" t="str">
         <f aca="false">IFERROR("FY"&amp;INDEX($C$47:$E$47,MATCH("BELOW",C58:E58,0)),"None")</f>
@@ -8960,12 +10307,12 @@
         <v>None</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>331</v>
+        <v>373</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>292</v>
+        <v>334</v>
       </c>
       <c r="C35" s="27" t="n">
         <f aca="false">SUM(C53:E53)</f>
@@ -8988,12 +10335,12 @@
         <v>-6882820.950603</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>332</v>
+        <v>374</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>293</v>
+        <v>335</v>
       </c>
       <c r="C36" s="28" t="n">
         <f aca="false">-AVERAGE(C53:E53)</f>
@@ -9016,12 +10363,12 @@
         <v>2294273.650201</v>
       </c>
       <c r="I36" s="26" t="s">
-        <v>333</v>
+        <v>375</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>334</v>
+        <v>376</v>
       </c>
       <c r="C37" s="27" t="n">
         <f aca="false">-AVERAGE(C53:E53)*$C$17</f>
@@ -9044,12 +10391,12 @@
         <v>9177094.600804</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>335</v>
+        <v>377</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>336</v>
+        <v>378</v>
       </c>
       <c r="C38" s="41" t="n">
         <f aca="false">-C53/C50</f>
@@ -9072,40 +10419,40 @@
         <v>0.291734458263779</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>337</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="C39" s="75" t="n">
+        <v>380</v>
+      </c>
+      <c r="C39" s="78" t="n">
         <f aca="false">IF(E53&lt;0,E56/-E53,"n/a")</f>
         <v>4.03903300374473</v>
       </c>
-      <c r="D39" s="75" t="n">
+      <c r="D39" s="78" t="n">
         <f aca="false">IF(E64&lt;0,E67/-E64,"n/a")</f>
         <v>2.88679052798419</v>
       </c>
-      <c r="E39" s="75" t="n">
+      <c r="E39" s="78" t="n">
         <f aca="false">IF(E75&lt;0,E78/-E75,"n/a")</f>
         <v>2.73224827727075</v>
       </c>
-      <c r="F39" s="75" t="n">
+      <c r="F39" s="78" t="n">
         <f aca="false">IF(E86&lt;0,E89/-E86,"n/a")</f>
         <v>7.48892133036166</v>
       </c>
-      <c r="G39" s="75" t="n">
+      <c r="G39" s="78" t="n">
         <f aca="false">IF(E97&lt;0,E100/-E97,"n/a")</f>
         <v>1.79391769362911</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>339</v>
+        <v>381</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>340</v>
+        <v>382</v>
       </c>
       <c r="C40" s="45" t="n">
         <f aca="false">(E56-SUM(C55:E55))/(E52/12)</f>
@@ -9128,12 +10475,12 @@
         <v>-0.60662708248183</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>341</v>
+        <v>383</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>342</v>
+        <v>384</v>
       </c>
       <c r="C41" s="45" t="n">
         <f aca="false">(E56+IF($C$23=1,MIN($C$24,Inputs!$G$37),Inputs!$G$37))/(E52/12)</f>
@@ -9156,12 +10503,12 @@
         <v>7.50804811696392</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>343</v>
+        <v>385</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>344</v>
+        <v>386</v>
       </c>
       <c r="C42" s="13" t="str">
         <f aca="false">IF(AND(ABS(INDEX(C31:G31,$C$6)-Forecast!E43)&lt;=1,ABS(INDEX(C32:G32,$C$6)-Forecast!E47)&lt;0.01),"OK","CHECK")</f>
@@ -9170,7 +10517,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>345</v>
+        <v>387</v>
       </c>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
@@ -9186,32 +10533,32 @@
         <v>9</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>346</v>
+        <v>388</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>246</v>
+        <v>289</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>247</v>
+        <v>290</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>248</v>
+        <v>291</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B47" s="53" t="n">
+        <v>293</v>
+      </c>
+      <c r="B47" s="56" t="n">
         <v>2025</v>
       </c>
-      <c r="C47" s="53" t="n">
+      <c r="C47" s="56" t="n">
         <v>2026</v>
       </c>
-      <c r="D47" s="53" t="n">
+      <c r="D47" s="56" t="n">
         <v>2027</v>
       </c>
-      <c r="E47" s="53" t="n">
+      <c r="E47" s="56" t="n">
         <v>2028</v>
       </c>
     </row>
@@ -9227,7 +10574,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="C50" s="27" t="n">
         <f aca="false">$C$11*(1+$C$12)^(C$47-$B$47)+$C$13*(1+$C$14)^(C$47-$B$47)+Forecast!$B$28*(1+$C$19)^(C$47-$B$47)+$C$20</f>
@@ -9244,7 +10591,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="C51" s="27" t="n">
         <f aca="false">IF(AND($C$15=1,MOD(C$47-$C$18,$C$17)=0),$C$16,0)</f>
@@ -9278,7 +10625,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>348</v>
+        <v>390</v>
       </c>
       <c r="C53" s="27" t="n">
         <f aca="false">C50-C52</f>
@@ -9295,7 +10642,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>349</v>
+        <v>391</v>
       </c>
       <c r="C54" s="27" t="n">
         <f aca="false">SUMPRODUCT($C51:C51*((C$47-$C$47:C$47)&lt;$C$17))/$C$17</f>
@@ -9312,7 +10659,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="C55" s="27" t="n">
         <f aca="false">IF(AND($C$23=1,(C$47-$B$47)&lt;=$C$25),MAX(0,Inputs!$G$37-$C$24)/$C$25,0)</f>
@@ -9329,7 +10676,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="B56" s="47" t="n">
         <f aca="false">Inputs!$G$36</f>
@@ -9356,22 +10703,22 @@
         <f aca="false">B56/(Forecast!$B$34/12)</f>
         <v>9.5070809221529</v>
       </c>
-      <c r="C57" s="61" t="n">
+      <c r="C57" s="64" t="n">
         <f aca="false">C56/(C52/12)</f>
         <v>9.41333881120348</v>
       </c>
-      <c r="D57" s="61" t="n">
+      <c r="D57" s="64" t="n">
         <f aca="false">D56/(D52/12)</f>
         <v>10.4866465289604</v>
       </c>
-      <c r="E57" s="61" t="n">
+      <c r="E57" s="64" t="n">
         <f aca="false">E56/(E52/12)</f>
         <v>10.9357207797708</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>351</v>
+        <v>393</v>
       </c>
       <c r="C58" s="19" t="str">
         <f aca="false">IF(C57&lt;$C$22,"BELOW","OK")</f>
@@ -9398,7 +10745,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="C61" s="27" t="n">
         <f aca="false">$D$11*(1+$D$12)^(C$47-$B$47)+$D$13*(1+$D$14)^(C$47-$B$47)+Forecast!$B$28*(1+$D$19)^(C$47-$B$47)+$D$20</f>
@@ -9415,7 +10762,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14" t="s">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="C62" s="27" t="n">
         <f aca="false">IF(AND($D$15=1,MOD(C$47-$D$18,$D$17)=0),$D$16,0)</f>
@@ -9449,7 +10796,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14" t="s">
-        <v>348</v>
+        <v>390</v>
       </c>
       <c r="C64" s="27" t="n">
         <f aca="false">C61-C63</f>
@@ -9466,7 +10813,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14" t="s">
-        <v>349</v>
+        <v>391</v>
       </c>
       <c r="C65" s="27" t="n">
         <f aca="false">SUMPRODUCT($C62:C62*((C$47-$C$47:C$47)&lt;$D$17))/$D$17</f>
@@ -9483,7 +10830,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="C66" s="27" t="n">
         <f aca="false">IF(AND($D$23=1,(C$47-$B$47)&lt;=$D$25),MAX(0,Inputs!$G$37-$D$24)/$D$25,0)</f>
@@ -9500,7 +10847,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="B67" s="47" t="n">
         <f aca="false">Inputs!$G$36</f>
@@ -9527,22 +10874,22 @@
         <f aca="false">B67/(Forecast!$B$34/12)</f>
         <v>9.5070809221529</v>
       </c>
-      <c r="C68" s="61" t="n">
+      <c r="C68" s="64" t="n">
         <f aca="false">C67/(C63/12)</f>
         <v>9.41333881120348</v>
       </c>
-      <c r="D68" s="61" t="n">
+      <c r="D68" s="64" t="n">
         <f aca="false">D67/(D63/12)</f>
         <v>8.83320149740756</v>
       </c>
-      <c r="E68" s="61" t="n">
+      <c r="E68" s="64" t="n">
         <f aca="false">E67/(E63/12)</f>
         <v>7.81601317306727</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14" t="s">
-        <v>351</v>
+        <v>393</v>
       </c>
       <c r="C69" s="19" t="str">
         <f aca="false">IF(C68&lt;$D$22,"BELOW","OK")</f>
@@ -9569,7 +10916,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="C72" s="27" t="n">
         <f aca="false">$E$11*(1+$E$12)^(C$47-$B$47)+$E$13*(1+$E$14)^(C$47-$B$47)+Forecast!$B$28*(1+$E$19)^(C$47-$B$47)+$E$20</f>
@@ -9586,7 +10933,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14" t="s">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="C73" s="27" t="n">
         <f aca="false">IF(AND($E$15=1,MOD(C$47-$E$18,$E$17)=0),$E$16,0)</f>
@@ -9620,7 +10967,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14" t="s">
-        <v>348</v>
+        <v>390</v>
       </c>
       <c r="C75" s="27" t="n">
         <f aca="false">C72-C74</f>
@@ -9637,7 +10984,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14" t="s">
-        <v>349</v>
+        <v>391</v>
       </c>
       <c r="C76" s="27" t="n">
         <f aca="false">SUMPRODUCT($C73:C73*((C$47-$C$47:C$47)&lt;$E$17))/$E$17</f>
@@ -9654,7 +11001,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="C77" s="27" t="n">
         <f aca="false">IF(AND($E$23=1,(C$47-$B$47)&lt;=$E$25),MAX(0,Inputs!$G$37-$E$24)/$E$25,0)</f>
@@ -9671,7 +11018,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="B78" s="47" t="n">
         <f aca="false">Inputs!$G$36</f>
@@ -9698,22 +11045,22 @@
         <f aca="false">B78/(Forecast!$B$34/12)</f>
         <v>9.5070809221529</v>
       </c>
-      <c r="C79" s="61" t="n">
+      <c r="C79" s="64" t="n">
         <f aca="false">C78/(C74/12)</f>
         <v>8.71981592240027</v>
       </c>
-      <c r="D79" s="61" t="n">
+      <c r="D79" s="64" t="n">
         <f aca="false">D78/(D74/12)</f>
         <v>9.17811277650154</v>
       </c>
-      <c r="E79" s="61" t="n">
+      <c r="E79" s="64" t="n">
         <f aca="false">E78/(E74/12)</f>
         <v>9.08402207346106</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14" t="s">
-        <v>351</v>
+        <v>393</v>
       </c>
       <c r="C80" s="19" t="str">
         <f aca="false">IF(C79&lt;$E$22,"BELOW","OK")</f>
@@ -9740,7 +11087,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="C83" s="27" t="n">
         <f aca="false">$F$11*(1+$F$12)^(C$47-$B$47)+$F$13*(1+$F$14)^(C$47-$B$47)+Forecast!$B$28*(1+$F$19)^(C$47-$B$47)+$F$20</f>
@@ -9757,7 +11104,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14" t="s">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="C84" s="27" t="n">
         <f aca="false">IF(AND($F$15=1,MOD(C$47-$F$18,$F$17)=0),$F$16,0)</f>
@@ -9791,7 +11138,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14" t="s">
-        <v>348</v>
+        <v>390</v>
       </c>
       <c r="C86" s="27" t="n">
         <f aca="false">C83-C85</f>
@@ -9808,7 +11155,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14" t="s">
-        <v>349</v>
+        <v>391</v>
       </c>
       <c r="C87" s="27" t="n">
         <f aca="false">SUMPRODUCT($C84:C84*((C$47-$C$47:C$47)&lt;$F$17))/$F$17</f>
@@ -9825,7 +11172,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="14" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="C88" s="27" t="n">
         <f aca="false">IF(AND($F$23=1,(C$47-$B$47)&lt;=$F$25),MAX(0,Inputs!$G$37-$F$24)/$F$25,0)</f>
@@ -9842,7 +11189,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="B89" s="47" t="n">
         <f aca="false">Inputs!$G$36</f>
@@ -9869,22 +11216,22 @@
         <f aca="false">B89/(Forecast!$B$34/12)</f>
         <v>9.5070809221529</v>
       </c>
-      <c r="C90" s="61" t="n">
+      <c r="C90" s="64" t="n">
         <f aca="false">C89/(C85/12)</f>
         <v>10.0370282911415</v>
       </c>
-      <c r="D90" s="61" t="n">
+      <c r="D90" s="64" t="n">
         <f aca="false">D89/(D85/12)</f>
         <v>12.1549590347252</v>
       </c>
-      <c r="E90" s="61" t="n">
+      <c r="E90" s="64" t="n">
         <f aca="false">E89/(E85/12)</f>
         <v>14.0167547980781</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>351</v>
+        <v>393</v>
       </c>
       <c r="C91" s="19" t="str">
         <f aca="false">IF(C90&lt;$F$22,"BELOW","OK")</f>
@@ -9911,7 +11258,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="C94" s="27" t="n">
         <f aca="false">$G$11*(1+$G$12)^(C$47-$B$47)+$G$13*(1+$G$14)^(C$47-$B$47)+Forecast!$B$28*(1+$G$19)^(C$47-$B$47)+$G$20</f>
@@ -9928,7 +11275,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14" t="s">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="C95" s="27" t="n">
         <f aca="false">IF(AND($G$15=1,MOD(C$47-$G$18,$G$17)=0),$G$16,0)</f>
@@ -9962,7 +11309,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14" t="s">
-        <v>348</v>
+        <v>390</v>
       </c>
       <c r="C97" s="27" t="n">
         <f aca="false">C94-C96</f>
@@ -9979,7 +11326,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14" t="s">
-        <v>349</v>
+        <v>391</v>
       </c>
       <c r="C98" s="27" t="n">
         <f aca="false">SUMPRODUCT($C95:C95*((C$47-$C$47:C$47)&lt;$G$17))/$G$17</f>
@@ -9996,7 +11343,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="C99" s="27" t="n">
         <f aca="false">IF(AND($G$23=1,(C$47-$B$47)&lt;=$G$25),MAX(0,Inputs!$G$37-$G$24)/$G$25,0)</f>
@@ -10013,7 +11360,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="B100" s="47" t="n">
         <f aca="false">Inputs!$G$36</f>
@@ -10040,22 +11387,22 @@
         <f aca="false">B100/(Forecast!$B$34/12)</f>
         <v>9.5070809221529</v>
       </c>
-      <c r="C101" s="61" t="n">
+      <c r="C101" s="64" t="n">
         <f aca="false">C100/(C96/12)</f>
         <v>8.71981592240027</v>
       </c>
-      <c r="D101" s="61" t="n">
+      <c r="D101" s="64" t="n">
         <f aca="false">D100/(D96/12)</f>
         <v>7.52466774494866</v>
       </c>
-      <c r="E101" s="61" t="n">
+      <c r="E101" s="64" t="n">
         <f aca="false">E100/(E96/12)</f>
         <v>5.9643144667575</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14" t="s">
-        <v>351</v>
+        <v>393</v>
       </c>
       <c r="C102" s="19" t="str">
         <f aca="false">IF(C101&lt;$G$22,"BELOW","OK")</f>

</xml_diff>